<commit_message>
Deleted all NCBI related code
</commit_message>
<xml_diff>
--- a/docs/data_providers/data_format/Example.xlsx
+++ b/docs/data_providers/data_format/Example.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jc2017/Documents/MyRepos/safedata_validator/docs/data_providers/data_format/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AE3DD28-562F-EF46-BB9F-5B8DE1CA9D52}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0D119B1-AA6D-9945-B9C3-17869DE5B1FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="500" windowWidth="27360" windowHeight="16940" xr2:uid="{958BE4CB-34F0-9B46-9A32-339A0F6D953C}"/>
+    <workbookView xWindow="360" yWindow="760" windowWidth="27360" windowHeight="16940" activeTab="6" xr2:uid="{958BE4CB-34F0-9B46-9A32-339A0F6D953C}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
     <sheet name="GBIFTaxa" sheetId="2" r:id="rId2"/>
-    <sheet name="NCBITaxa" sheetId="3" r:id="rId3"/>
+    <sheet name="SeqTaxa" sheetId="3" r:id="rId3"/>
     <sheet name="Locations" sheetId="4" r:id="rId4"/>
     <sheet name="abundances_1" sheetId="5" r:id="rId5"/>
     <sheet name="abundances_2" sheetId="6" r:id="rId6"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="260">
   <si>
     <t>Title</t>
   </si>
@@ -274,9 +274,6 @@
     <t>New</t>
   </si>
   <si>
-    <t>Superkingdom</t>
-  </si>
-  <si>
     <t>Kingdom</t>
   </si>
   <si>
@@ -286,57 +283,9 @@
     <t>Class</t>
   </si>
   <si>
-    <t>G_proteobacteria</t>
-  </si>
-  <si>
-    <t>Bacteria</t>
-  </si>
-  <si>
-    <t>Pseudomonadota</t>
-  </si>
-  <si>
-    <t>Gammaproteobacteria</t>
-  </si>
-  <si>
-    <t>E_mycetes</t>
-  </si>
-  <si>
-    <t>Eukaryota</t>
-  </si>
-  <si>
-    <t>Fungi</t>
-  </si>
-  <si>
-    <t>Ascomycota</t>
-  </si>
-  <si>
-    <t>Eurotiomycetes</t>
-  </si>
-  <si>
-    <t>Dinophyceae</t>
-  </si>
-  <si>
-    <t>Acidobact</t>
-  </si>
-  <si>
-    <t>k__Bacteria</t>
-  </si>
-  <si>
-    <t>p__Acidobacteria</t>
-  </si>
-  <si>
-    <t>c__Acidobacteriia</t>
-  </si>
-  <si>
-    <t>New_fungus</t>
-  </si>
-  <si>
     <t>Yes</t>
   </si>
   <si>
-    <t>Mynewfungusetes</t>
-  </si>
-  <si>
     <t>Location name</t>
   </si>
   <si>
@@ -674,6 +623,198 @@
   </si>
   <si>
     <t>A second raster file containing altitudes</t>
+  </si>
+  <si>
+    <t>Order</t>
+  </si>
+  <si>
+    <t>ASV_100</t>
+  </si>
+  <si>
+    <t>k__Fungi</t>
+  </si>
+  <si>
+    <t>p__Basidiomycota</t>
+  </si>
+  <si>
+    <t>c__Tremellomycetes</t>
+  </si>
+  <si>
+    <t>o__Tremellales</t>
+  </si>
+  <si>
+    <t>f__Trimorphomycetaceae</t>
+  </si>
+  <si>
+    <t>g__Saitozyma</t>
+  </si>
+  <si>
+    <t>s__podzolica</t>
+  </si>
+  <si>
+    <t>ASV_101</t>
+  </si>
+  <si>
+    <t>p__Ascomycota</t>
+  </si>
+  <si>
+    <t>c__Sordariomycetes</t>
+  </si>
+  <si>
+    <t>o__Hypocreales</t>
+  </si>
+  <si>
+    <t>f__Hypocreaceae</t>
+  </si>
+  <si>
+    <t>g__Trichoderma</t>
+  </si>
+  <si>
+    <t>s__spirale</t>
+  </si>
+  <si>
+    <t>ASV_102</t>
+  </si>
+  <si>
+    <t>o__Trichosporonales</t>
+  </si>
+  <si>
+    <t>f__Trichosporonaceae</t>
+  </si>
+  <si>
+    <t>g__Apiotrichum</t>
+  </si>
+  <si>
+    <t>s__sporotrichoides</t>
+  </si>
+  <si>
+    <t>ASV_103</t>
+  </si>
+  <si>
+    <t>ASV_104</t>
+  </si>
+  <si>
+    <t>p__Mortierellomycota</t>
+  </si>
+  <si>
+    <t>c__Mortierellomycetes</t>
+  </si>
+  <si>
+    <t>o__Mortierellales</t>
+  </si>
+  <si>
+    <t>f__Mortierellaceae</t>
+  </si>
+  <si>
+    <t>g__Mortierella</t>
+  </si>
+  <si>
+    <t>s__elongata</t>
+  </si>
+  <si>
+    <t>ASV_105</t>
+  </si>
+  <si>
+    <t>c__Eurotiomycetes</t>
+  </si>
+  <si>
+    <t>o__Eurotiales</t>
+  </si>
+  <si>
+    <t>f__Trichocomaceae</t>
+  </si>
+  <si>
+    <t>g__Talaromyces</t>
+  </si>
+  <si>
+    <t>ASV_106</t>
+  </si>
+  <si>
+    <t>f__Ophiocordycipitaceae</t>
+  </si>
+  <si>
+    <t>g__Purpureocillium</t>
+  </si>
+  <si>
+    <t>s__lilacinum</t>
+  </si>
+  <si>
+    <t>ASV_107</t>
+  </si>
+  <si>
+    <t>s__harzianum</t>
+  </si>
+  <si>
+    <t>ASV_108</t>
+  </si>
+  <si>
+    <t>c__Geoglossomycetes</t>
+  </si>
+  <si>
+    <t>o__Geoglossales</t>
+  </si>
+  <si>
+    <t>f__Geoglossaceae</t>
+  </si>
+  <si>
+    <t>g__Geoglossum</t>
+  </si>
+  <si>
+    <t>s__difforme</t>
+  </si>
+  <si>
+    <t>ASV_109</t>
+  </si>
+  <si>
+    <t>Example comment</t>
+  </si>
+  <si>
+    <t>ASV_110</t>
+  </si>
+  <si>
+    <t>c__Dothideomycetes</t>
+  </si>
+  <si>
+    <t>o__Pleosporales</t>
+  </si>
+  <si>
+    <t>f__Cucurbitariaceae</t>
+  </si>
+  <si>
+    <t>g__Pyrenochaetopsis</t>
+  </si>
+  <si>
+    <t>s__leptospora</t>
+  </si>
+  <si>
+    <t>ASV_111</t>
+  </si>
+  <si>
+    <t>s__koningiopsis</t>
+  </si>
+  <si>
+    <t>ASV_113</t>
+  </si>
+  <si>
+    <t>f__Clavicipitaceae</t>
+  </si>
+  <si>
+    <t>g__Metarhizium</t>
+  </si>
+  <si>
+    <t>s__carneum</t>
+  </si>
+  <si>
+    <t>ASV_114</t>
+  </si>
+  <si>
+    <t>o__Chaetosphaeriales</t>
+  </si>
+  <si>
+    <t>f__Chaetosphaeriaceae</t>
+  </si>
+  <si>
+    <t>g__Chloridium</t>
   </si>
 </sst>
 </file>
@@ -730,8 +871,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -751,9 +894,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -791,7 +934,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -897,7 +1040,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1039,7 +1182,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1139,25 +1282,25 @@
         <v>17</v>
       </c>
       <c r="B11" t="s">
-        <v>182</v>
+        <v>165</v>
       </c>
       <c r="C11" t="s">
-        <v>184</v>
+        <v>167</v>
       </c>
       <c r="D11" t="s">
-        <v>188</v>
+        <v>171</v>
       </c>
       <c r="E11" t="s">
-        <v>189</v>
+        <v>172</v>
       </c>
       <c r="F11" t="s">
-        <v>190</v>
+        <v>173</v>
       </c>
       <c r="G11" t="s">
-        <v>197</v>
+        <v>180</v>
       </c>
       <c r="H11" t="s">
-        <v>198</v>
+        <v>181</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
@@ -1165,51 +1308,51 @@
         <v>18</v>
       </c>
       <c r="B12" t="s">
+        <v>166</v>
+      </c>
+      <c r="C12" t="s">
+        <v>168</v>
+      </c>
+      <c r="D12" t="s">
+        <v>174</v>
+      </c>
+      <c r="E12" t="s">
+        <v>175</v>
+      </c>
+      <c r="F12" t="s">
+        <v>176</v>
+      </c>
+      <c r="G12" t="s">
+        <v>182</v>
+      </c>
+      <c r="H12" t="s">
         <v>183</v>
-      </c>
-      <c r="C12" t="s">
-        <v>185</v>
-      </c>
-      <c r="D12" t="s">
-        <v>191</v>
-      </c>
-      <c r="E12" t="s">
-        <v>192</v>
-      </c>
-      <c r="F12" t="s">
-        <v>193</v>
-      </c>
-      <c r="G12" t="s">
-        <v>199</v>
-      </c>
-      <c r="H12" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>160</v>
+      </c>
+      <c r="B13" t="s">
+        <v>170</v>
+      </c>
+      <c r="C13" t="s">
+        <v>169</v>
+      </c>
+      <c r="D13" t="s">
         <v>177</v>
       </c>
-      <c r="B13" t="s">
-        <v>187</v>
-      </c>
-      <c r="C13" t="s">
-        <v>186</v>
-      </c>
-      <c r="D13" t="s">
-        <v>194</v>
-      </c>
       <c r="E13" t="s">
-        <v>195</v>
+        <v>178</v>
       </c>
       <c r="F13" t="s">
-        <v>196</v>
+        <v>179</v>
       </c>
       <c r="G13" t="s">
-        <v>202</v>
+        <v>185</v>
       </c>
       <c r="H13" t="s">
-        <v>201</v>
+        <v>184</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
@@ -1236,24 +1379,24 @@
         <v>46</v>
       </c>
       <c r="C16" t="s">
-        <v>166</v>
+        <v>149</v>
       </c>
       <c r="D16" t="s">
-        <v>167</v>
+        <v>150</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>178</v>
+        <v>161</v>
       </c>
       <c r="B17" t="s">
         <v>47</v>
       </c>
       <c r="C17" t="s">
-        <v>212</v>
+        <v>195</v>
       </c>
       <c r="D17" t="s">
-        <v>211</v>
+        <v>194</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
@@ -1388,149 +1531,145 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>159</v>
+      <c r="A1" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B1" t="s">
+        <v>141</v>
+      </c>
+      <c r="C1" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>161</v>
+      <c r="A2" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C2" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="C3" s="3"/>
+      <c r="A3" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B3" t="s">
+        <v>145</v>
+      </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
+      <c r="A4" s="3" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="C5" s="3"/>
+      <c r="A5" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B5" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>165</v>
+      <c r="A6" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B6" t="s">
+        <v>147</v>
+      </c>
+      <c r="C6" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" s="4">
+      <c r="A7" s="3">
         <v>1</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7">
         <v>100</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>166</v>
+      <c r="C7" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" s="4">
+      <c r="A8" s="3">
         <v>2</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8">
         <v>200</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>166</v>
+      <c r="C8" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" s="4">
+      <c r="A9" s="3">
         <v>3</v>
       </c>
-      <c r="B9" s="3">
+      <c r="B9">
         <v>300</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>166</v>
+      <c r="C9" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" s="4">
+      <c r="A10" s="3">
         <v>4</v>
       </c>
-      <c r="B10" s="3">
+      <c r="B10">
         <v>400</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>166</v>
+      <c r="C10" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" s="4">
+      <c r="A11" s="3">
         <v>5</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B11">
         <v>500</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>167</v>
+      <c r="C11" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" s="4">
+      <c r="A12" s="3">
         <v>6</v>
       </c>
-      <c r="B12" s="3">
+      <c r="B12">
         <v>600</v>
       </c>
-      <c r="C12" s="3" t="s">
-        <v>167</v>
+      <c r="C12" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" s="4">
+      <c r="A13" s="3">
         <v>7</v>
       </c>
-      <c r="B13" s="3">
+      <c r="B13">
         <v>700</v>
       </c>
-      <c r="C13" s="3" t="s">
-        <v>167</v>
+      <c r="C13" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A14" s="4">
+      <c r="A14" s="3">
         <v>8</v>
       </c>
-      <c r="B14" s="3">
+      <c r="B14">
         <v>800</v>
       </c>
-      <c r="C14" s="3" t="s">
-        <v>167</v>
+      <c r="C14" t="s">
+        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -1549,158 +1688,153 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="B1" s="3" t="s">
+      <c r="A1" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B1" t="s">
+        <v>141</v>
+      </c>
+      <c r="C1" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C2" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B5" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="C6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B7" t="s">
+        <v>147</v>
+      </c>
+      <c r="C7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="3">
+        <v>1</v>
+      </c>
+      <c r="B8">
+        <v>100</v>
+      </c>
+      <c r="C8" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="3">
+        <v>2</v>
+      </c>
+      <c r="B9">
+        <v>200</v>
+      </c>
+      <c r="C9" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="3">
+        <v>3</v>
+      </c>
+      <c r="B10">
+        <v>300</v>
+      </c>
+      <c r="C10" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" s="3">
+        <v>4</v>
+      </c>
+      <c r="B11">
+        <v>400</v>
+      </c>
+      <c r="C11" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" s="3">
+        <v>5</v>
+      </c>
+      <c r="B12">
+        <v>500</v>
+      </c>
+      <c r="C12" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" s="3">
+        <v>6</v>
+      </c>
+      <c r="B13">
+        <v>600</v>
+      </c>
+      <c r="C13" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" s="3">
+        <v>7</v>
+      </c>
+      <c r="B14">
+        <v>700</v>
+      </c>
+      <c r="C14" t="s">
         <v>158</v>
       </c>
-      <c r="C1" s="3" t="s">
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" s="3">
+        <v>8</v>
+      </c>
+      <c r="B15">
+        <v>800</v>
+      </c>
+      <c r="C15" t="s">
         <v>159</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="C3" s="3"/>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="C5" s="3"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" s="4">
-        <v>1</v>
-      </c>
-      <c r="B8" s="3">
-        <v>100</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" s="4">
-        <v>2</v>
-      </c>
-      <c r="B9" s="3">
-        <v>200</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" s="4">
-        <v>3</v>
-      </c>
-      <c r="B10" s="3">
-        <v>300</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" s="4">
-        <v>4</v>
-      </c>
-      <c r="B11" s="3">
-        <v>400</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" s="4">
-        <v>5</v>
-      </c>
-      <c r="B12" s="3">
-        <v>500</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" s="4">
-        <v>6</v>
-      </c>
-      <c r="B13" s="3">
-        <v>600</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A14" s="4">
-        <v>7</v>
-      </c>
-      <c r="B14" s="3">
-        <v>700</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A15" s="4">
-        <v>8</v>
-      </c>
-      <c r="B15" s="3">
-        <v>800</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>176</v>
       </c>
     </row>
   </sheetData>
@@ -1723,242 +1857,213 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A1" s="3" t="s">
+      <c r="A1" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" t="s">
         <v>49</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" t="s">
         <v>50</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" t="s">
         <v>51</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" t="s">
         <v>52</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" t="s">
         <v>54</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" t="s">
         <v>53</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" t="s">
         <v>55</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" t="s">
         <v>57</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" t="s">
         <v>58</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" t="s">
         <v>59</v>
       </c>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
+      <c r="A3" t="s">
         <v>60</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" t="s">
         <v>61</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" t="s">
         <v>62</v>
       </c>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
+      <c r="A4" t="s">
         <v>63</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" t="s">
         <v>64</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" t="s">
         <v>62</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4">
         <v>2480962</v>
       </c>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
+      <c r="A5" t="s">
         <v>65</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" t="s">
         <v>66</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" t="s">
         <v>59</v>
       </c>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3" t="s">
+      <c r="F5" t="s">
         <v>67</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" t="s">
         <v>62</v>
       </c>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3" t="s">
+      <c r="I5" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
+      <c r="A6" t="s">
         <v>69</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" t="s">
         <v>70</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" t="s">
         <v>71</v>
       </c>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3" t="s">
+      <c r="F6" t="s">
         <v>72</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G6" t="s">
         <v>73</v>
       </c>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
+      <c r="A7" t="s">
         <v>74</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" t="s">
         <v>75</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" t="s">
         <v>76</v>
       </c>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3" t="s">
+      <c r="F7" t="s">
         <v>77</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="G7" t="s">
         <v>73</v>
       </c>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="C8" s="3" t="s">
+      <c r="A8" t="s">
+        <v>163</v>
+      </c>
+      <c r="B8" t="s">
+        <v>162</v>
+      </c>
+      <c r="C8" t="s">
         <v>59</v>
       </c>
-      <c r="D8" s="3"/>
       <c r="E8">
         <v>5361886</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="F8" t="s">
         <v>64</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="G8" t="s">
         <v>62</v>
       </c>
-      <c r="H8" s="3">
+      <c r="H8">
         <v>2480962</v>
       </c>
-      <c r="I8" s="3" t="s">
-        <v>181</v>
+      <c r="I8" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>203</v>
-      </c>
-      <c r="C9" s="3" t="s">
+      <c r="A9" t="s">
+        <v>102</v>
+      </c>
+      <c r="B9" t="s">
+        <v>186</v>
+      </c>
+      <c r="C9" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A10" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="C10" s="3" t="s">
+      <c r="A10" t="s">
+        <v>103</v>
+      </c>
+      <c r="B10" t="s">
+        <v>187</v>
+      </c>
+      <c r="C10" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A11" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="C11" s="3" t="s">
+      <c r="A11" t="s">
+        <v>131</v>
+      </c>
+      <c r="B11" t="s">
+        <v>188</v>
+      </c>
+      <c r="C11" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A12" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>206</v>
-      </c>
-      <c r="C12" s="3" t="s">
+      <c r="A12" t="s">
+        <v>134</v>
+      </c>
+      <c r="B12" t="s">
+        <v>189</v>
+      </c>
+      <c r="C12" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A13" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>207</v>
-      </c>
-      <c r="C13" s="3" t="s">
+      <c r="A13" t="s">
+        <v>132</v>
+      </c>
+      <c r="B13" t="s">
+        <v>190</v>
+      </c>
+      <c r="C13" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A14" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>208</v>
-      </c>
-      <c r="C14" s="3" t="s">
+      <c r="A14" t="s">
+        <v>135</v>
+      </c>
+      <c r="B14" t="s">
+        <v>191</v>
+      </c>
+      <c r="C14" t="s">
         <v>59</v>
       </c>
     </row>
@@ -1969,127 +2074,412 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95D2376D-CAF7-794F-A21C-41734DBF2E1E}">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.1640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.5" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="21.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>48</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>81</v>
+        <v>196</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="G1" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="I1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="G2" s="3"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="G3" s="3"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="G4" s="3"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="G5" s="3"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="G6" s="3"/>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>197</v>
+      </c>
+      <c r="B2" t="s">
+        <v>198</v>
+      </c>
+      <c r="C2" t="s">
+        <v>199</v>
+      </c>
+      <c r="D2" t="s">
+        <v>200</v>
+      </c>
+      <c r="E2" t="s">
+        <v>201</v>
+      </c>
+      <c r="F2" t="s">
+        <v>202</v>
+      </c>
+      <c r="G2" t="s">
+        <v>203</v>
+      </c>
+      <c r="H2" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>205</v>
+      </c>
+      <c r="B3" t="s">
+        <v>198</v>
+      </c>
+      <c r="C3" t="s">
+        <v>206</v>
+      </c>
+      <c r="D3" t="s">
+        <v>207</v>
+      </c>
+      <c r="E3" t="s">
+        <v>208</v>
+      </c>
+      <c r="F3" t="s">
+        <v>209</v>
+      </c>
+      <c r="G3" t="s">
+        <v>210</v>
+      </c>
+      <c r="H3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>212</v>
+      </c>
+      <c r="B4" t="s">
+        <v>198</v>
+      </c>
+      <c r="C4" t="s">
+        <v>199</v>
+      </c>
+      <c r="D4" t="s">
+        <v>200</v>
+      </c>
+      <c r="E4" t="s">
+        <v>213</v>
+      </c>
+      <c r="F4" t="s">
+        <v>214</v>
+      </c>
+      <c r="G4" t="s">
+        <v>215</v>
+      </c>
+      <c r="H4" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>217</v>
+      </c>
+      <c r="B5" t="s">
+        <v>198</v>
+      </c>
+      <c r="C5" t="s">
+        <v>206</v>
+      </c>
+      <c r="D5" t="s">
+        <v>207</v>
+      </c>
+      <c r="E5" t="s">
+        <v>208</v>
+      </c>
+      <c r="F5" t="s">
+        <v>209</v>
+      </c>
+      <c r="G5" t="s">
+        <v>210</v>
+      </c>
+      <c r="H5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>218</v>
+      </c>
+      <c r="B6" t="s">
+        <v>198</v>
+      </c>
+      <c r="C6" t="s">
+        <v>219</v>
+      </c>
+      <c r="D6" t="s">
+        <v>220</v>
+      </c>
+      <c r="E6" t="s">
+        <v>221</v>
+      </c>
+      <c r="F6" t="s">
+        <v>222</v>
+      </c>
+      <c r="G6" t="s">
+        <v>223</v>
+      </c>
+      <c r="H6" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>225</v>
+      </c>
+      <c r="B7" t="s">
+        <v>198</v>
+      </c>
+      <c r="C7" t="s">
+        <v>206</v>
+      </c>
+      <c r="D7" t="s">
+        <v>226</v>
+      </c>
+      <c r="E7" t="s">
+        <v>227</v>
+      </c>
+      <c r="F7" t="s">
+        <v>228</v>
+      </c>
+      <c r="G7" t="s">
+        <v>229</v>
+      </c>
+      <c r="H7" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>230</v>
+      </c>
+      <c r="B8" t="s">
+        <v>198</v>
+      </c>
+      <c r="C8" t="s">
+        <v>206</v>
+      </c>
+      <c r="D8" t="s">
+        <v>207</v>
+      </c>
+      <c r="E8" t="s">
+        <v>208</v>
+      </c>
+      <c r="F8" t="s">
+        <v>231</v>
+      </c>
+      <c r="G8" t="s">
+        <v>232</v>
+      </c>
+      <c r="H8" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>234</v>
+      </c>
+      <c r="B9" t="s">
+        <v>198</v>
+      </c>
+      <c r="C9" t="s">
+        <v>206</v>
+      </c>
+      <c r="D9" t="s">
+        <v>207</v>
+      </c>
+      <c r="E9" t="s">
+        <v>208</v>
+      </c>
+      <c r="F9" t="s">
+        <v>209</v>
+      </c>
+      <c r="G9" t="s">
+        <v>210</v>
+      </c>
+      <c r="H9" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>236</v>
+      </c>
+      <c r="B10" t="s">
+        <v>198</v>
+      </c>
+      <c r="C10" t="s">
+        <v>206</v>
+      </c>
+      <c r="D10" t="s">
+        <v>237</v>
+      </c>
+      <c r="E10" t="s">
+        <v>238</v>
+      </c>
+      <c r="F10" t="s">
+        <v>239</v>
+      </c>
+      <c r="G10" t="s">
+        <v>240</v>
+      </c>
+      <c r="H10" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>242</v>
+      </c>
+      <c r="B11" t="s">
+        <v>198</v>
+      </c>
+      <c r="C11" t="s">
+        <v>206</v>
+      </c>
+      <c r="D11" t="s">
+        <v>207</v>
+      </c>
+      <c r="E11" t="s">
+        <v>208</v>
+      </c>
+      <c r="F11" t="s">
+        <v>209</v>
+      </c>
+      <c r="G11" t="s">
+        <v>210</v>
+      </c>
+      <c r="H11" t="s">
+        <v>235</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>244</v>
+      </c>
+      <c r="B12" t="s">
+        <v>198</v>
+      </c>
+      <c r="C12" t="s">
+        <v>206</v>
+      </c>
+      <c r="D12" t="s">
+        <v>245</v>
+      </c>
+      <c r="E12" t="s">
+        <v>246</v>
+      </c>
+      <c r="F12" t="s">
+        <v>247</v>
+      </c>
+      <c r="G12" t="s">
+        <v>248</v>
+      </c>
+      <c r="H12" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>250</v>
+      </c>
+      <c r="B13" t="s">
+        <v>198</v>
+      </c>
+      <c r="C13" t="s">
+        <v>206</v>
+      </c>
+      <c r="D13" t="s">
+        <v>207</v>
+      </c>
+      <c r="E13" t="s">
+        <v>208</v>
+      </c>
+      <c r="F13" t="s">
+        <v>209</v>
+      </c>
+      <c r="G13" t="s">
+        <v>210</v>
+      </c>
+      <c r="H13" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>252</v>
+      </c>
+      <c r="B14" t="s">
+        <v>198</v>
+      </c>
+      <c r="C14" t="s">
+        <v>206</v>
+      </c>
+      <c r="D14" t="s">
+        <v>207</v>
+      </c>
+      <c r="E14" t="s">
+        <v>208</v>
+      </c>
+      <c r="F14" t="s">
+        <v>253</v>
+      </c>
+      <c r="G14" t="s">
+        <v>254</v>
+      </c>
+      <c r="H14" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>256</v>
+      </c>
+      <c r="B15" t="s">
+        <v>198</v>
+      </c>
+      <c r="C15" t="s">
+        <v>206</v>
+      </c>
+      <c r="D15" t="s">
+        <v>207</v>
+      </c>
+      <c r="E15" t="s">
+        <v>257</v>
+      </c>
+      <c r="F15" t="s">
+        <v>258</v>
+      </c>
+      <c r="G15" t="s">
+        <v>259</v>
+      </c>
+      <c r="H15" t="s">
+        <v>70</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2110,127 +2500,119 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="B1" s="3" t="s">
+      <c r="A1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B1" t="s">
         <v>78</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>104</v>
+      <c r="C1" t="s">
+        <v>84</v>
+      </c>
+      <c r="D1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E1" t="s">
+        <v>86</v>
+      </c>
+      <c r="F1" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
+      <c r="A2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
+      <c r="A3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B3" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="B4" s="3" t="s">
+      <c r="A4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C4">
+        <v>4.9577210000000003</v>
+      </c>
+      <c r="D4">
+        <v>117.776023</v>
+      </c>
+      <c r="E4" t="s">
+        <v>92</v>
+      </c>
+      <c r="F4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>93</v>
+      </c>
+      <c r="B5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C5" t="s">
+        <v>70</v>
+      </c>
+      <c r="D5" t="s">
+        <v>70</v>
+      </c>
+      <c r="E5" t="s">
+        <v>92</v>
+      </c>
+      <c r="F5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>94</v>
+      </c>
+      <c r="B6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C6" t="s">
+        <v>70</v>
+      </c>
+      <c r="D6" t="s">
+        <v>70</v>
+      </c>
+      <c r="E6" t="s">
+        <v>92</v>
+      </c>
+      <c r="F6" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B7" t="s">
+        <v>82</v>
+      </c>
+      <c r="C7" t="s">
+        <v>70</v>
+      </c>
+      <c r="D7" t="s">
+        <v>70</v>
+      </c>
+      <c r="E7" t="s">
+        <v>97</v>
+      </c>
+      <c r="F7" t="s">
         <v>98</v>
-      </c>
-      <c r="C4" s="3">
-        <v>4.9577210000000003</v>
-      </c>
-      <c r="D4" s="3">
-        <v>117.776023</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -2240,137 +2622,99 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7FB2131-D12F-E446-A544-0D39287054FC}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="3" width="30.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="D1" s="3"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="D2" s="3"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="D3" s="3"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="D4" s="3"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="D5" s="3"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="D6" s="3"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B4" t="s">
+        <v>107</v>
+      </c>
+      <c r="C4" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B5" t="s">
+        <v>109</v>
+      </c>
+      <c r="C5" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C6" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" s="3">
         <v>1</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7">
         <v>24</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7">
         <v>12</v>
       </c>
-      <c r="D7" s="3"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="4">
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="3">
         <v>2</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8">
         <v>62</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8">
         <v>3</v>
       </c>
-      <c r="D8" s="3"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2388,106 +2732,103 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="C3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B4" t="s">
         <v>116</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="C1" s="3" t="s">
+      <c r="C4" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>134</v>
-      </c>
-    </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3" t="s">
-        <v>126</v>
+      <c r="A5" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="C5" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>135</v>
+      <c r="A6" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B6" t="s">
+        <v>115</v>
+      </c>
+      <c r="C6" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" s="4">
+      <c r="A7" s="3">
         <v>1</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="C7" s="3">
+      <c r="B7" t="s">
+        <v>102</v>
+      </c>
+      <c r="C7">
         <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" s="4">
+      <c r="A8" s="3">
         <v>2</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C8" s="3">
+      <c r="B8" t="s">
+        <v>103</v>
+      </c>
+      <c r="C8">
         <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" s="4">
+      <c r="A9" s="3">
         <v>3</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="C9" s="3">
+      <c r="B9" t="s">
+        <v>102</v>
+      </c>
+      <c r="C9">
         <v>62</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" s="4">
+      <c r="A10" s="3">
         <v>4</v>
       </c>
-      <c r="B10" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C10" s="3">
+      <c r="B10" t="s">
+        <v>103</v>
+      </c>
+      <c r="C10">
         <v>3</v>
       </c>
     </row>
@@ -2507,107 +2848,103 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="B1" s="3" t="s">
+      <c r="A1" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C1" t="s">
+        <v>113</v>
+      </c>
+      <c r="D1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D3" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D4" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B5" t="s">
+        <v>125</v>
+      </c>
+      <c r="C5" t="s">
+        <v>126</v>
+      </c>
+      <c r="D5" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B6" t="s">
+        <v>128</v>
+      </c>
+      <c r="C6" t="s">
+        <v>129</v>
+      </c>
+      <c r="D6" t="s">
         <v>130</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="D1" s="3" t="s">
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" s="3">
+        <v>1</v>
+      </c>
+      <c r="B7" t="s">
+        <v>131</v>
+      </c>
+      <c r="C7" t="s">
+        <v>132</v>
+      </c>
+      <c r="D7" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" s="3">
+        <v>2</v>
+      </c>
+      <c r="B8" t="s">
+        <v>134</v>
+      </c>
+      <c r="C8" t="s">
+        <v>135</v>
+      </c>
+      <c r="D8" t="s">
         <v>136</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="4">
-        <v>1</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="4">
-        <v>2</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>153</v>
       </c>
     </row>
   </sheetData>
@@ -2625,67 +2962,67 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="B1" s="3" t="s">
+      <c r="A1" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="B2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B3" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B4" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B5" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B6" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" s="3">
+        <v>1</v>
+      </c>
+      <c r="B7" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" s="3">
+        <v>2</v>
+      </c>
+      <c r="B8" t="s">
         <v>136</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" s="4">
-        <v>1</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" s="4">
-        <v>2</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>153</v>
       </c>
     </row>
   </sheetData>
@@ -2704,96 +3041,93 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="B1" s="3" t="s">
+      <c r="A1" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="C2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C3" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C4" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C5" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B6" t="s">
+        <v>126</v>
+      </c>
+      <c r="C6" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B7" t="s">
+        <v>129</v>
+      </c>
+      <c r="C7" t="s">
         <v>130</v>
       </c>
-      <c r="C1" s="3" t="s">
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="3">
+        <v>1</v>
+      </c>
+      <c r="B8" t="s">
+        <v>132</v>
+      </c>
+      <c r="C8" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="3">
+        <v>2</v>
+      </c>
+      <c r="B9" t="s">
+        <v>135</v>
+      </c>
+      <c r="C9" t="s">
         <v>136</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" s="4">
-        <v>1</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" s="4">
-        <v>2</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>153</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added reading of sequenced taxa from multiple sheets
</commit_message>
<xml_diff>
--- a/docs/data_providers/data_format/Example.xlsx
+++ b/docs/data_providers/data_format/Example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jc2017/Documents/MyRepos/safedata_validator/docs/data_providers/data_format/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0D119B1-AA6D-9945-B9C3-17869DE5B1FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72DF311B-7C8F-6B49-B7B8-7AD70020ED90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="760" windowWidth="27360" windowHeight="16940" activeTab="6" xr2:uid="{958BE4CB-34F0-9B46-9A32-339A0F6D953C}"/>
+    <workbookView xWindow="360" yWindow="760" windowWidth="27360" windowHeight="16940" xr2:uid="{958BE4CB-34F0-9B46-9A32-339A0F6D953C}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="268">
   <si>
     <t>Title</t>
   </si>
@@ -815,6 +815,30 @@
   </si>
   <si>
     <t>g__Chloridium</t>
+  </si>
+  <si>
+    <t>Sequenced taxa sheet name</t>
+  </si>
+  <si>
+    <t>SeqTaxa</t>
+  </si>
+  <si>
+    <t>Reference database name</t>
+  </si>
+  <si>
+    <t>Greengenes</t>
+  </si>
+  <si>
+    <t>Reference database version</t>
+  </si>
+  <si>
+    <t>v1.7.9</t>
+  </si>
+  <si>
+    <t>Reference database link</t>
+  </si>
+  <si>
+    <t>https://greengenes2.ucsd.edu</t>
   </si>
 </sst>
 </file>
@@ -1190,10 +1214,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56835824-9479-A543-9F3B-4D7006FD1F4E}">
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="42.5" customWidth="1"/>
     <col min="3" max="3" width="23.1640625" bestFit="1" customWidth="1"/>
     <col min="4" max="6" width="20" bestFit="1" customWidth="1"/>
@@ -1511,11 +1535,44 @@
         <v>116.75</v>
       </c>
     </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>260</v>
+      </c>
+      <c r="B32" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>262</v>
+      </c>
+      <c r="B33" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>264</v>
+      </c>
+      <c r="B34" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>266</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>267</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B8" r:id="rId1" xr:uid="{8F2F57F5-1AEE-0D48-93D7-9691DA786243}"/>
     <hyperlink ref="B18" r:id="rId2" xr:uid="{854E441D-2155-F243-9B6D-EA2BAFB9B5A2}"/>
     <hyperlink ref="B22" r:id="rId3" xr:uid="{1F970723-7B44-4944-98C3-9AB1AB233E97}"/>
+    <hyperlink ref="B35" r:id="rId4" xr:uid="{3C58A218-390F-B04E-B352-36685BA79647}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated the documentation to explain how the multiple SeqTaxa sheets system works
</commit_message>
<xml_diff>
--- a/docs/data_providers/data_format/Example.xlsx
+++ b/docs/data_providers/data_format/Example.xlsx
@@ -8,22 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jc2017/Documents/MyRepos/safedata_validator/docs/data_providers/data_format/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72DF311B-7C8F-6B49-B7B8-7AD70020ED90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE15D25A-463D-3742-B77C-CB752AC55F80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="760" windowWidth="27360" windowHeight="16940" xr2:uid="{958BE4CB-34F0-9B46-9A32-339A0F6D953C}"/>
+    <workbookView xWindow="360" yWindow="760" windowWidth="27360" windowHeight="16940" activeTab="3" xr2:uid="{958BE4CB-34F0-9B46-9A32-339A0F6D953C}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
     <sheet name="GBIFTaxa" sheetId="2" r:id="rId2"/>
-    <sheet name="SeqTaxa" sheetId="3" r:id="rId3"/>
-    <sheet name="Locations" sheetId="4" r:id="rId4"/>
-    <sheet name="abundances_1" sheetId="5" r:id="rId5"/>
-    <sheet name="abundances_2" sheetId="6" r:id="rId6"/>
-    <sheet name="interactions_1" sheetId="7" r:id="rId7"/>
-    <sheet name="interactions_2" sheetId="8" r:id="rId8"/>
-    <sheet name="interactions_3" sheetId="9" r:id="rId9"/>
-    <sheet name="external_1" sheetId="10" r:id="rId10"/>
-    <sheet name="external_2" sheetId="11" r:id="rId11"/>
+    <sheet name="Sequenced" sheetId="3" r:id="rId3"/>
+    <sheet name="MoreSeqData" sheetId="12" r:id="rId4"/>
+    <sheet name="Locations" sheetId="4" r:id="rId5"/>
+    <sheet name="abundances_1" sheetId="5" r:id="rId6"/>
+    <sheet name="abundances_2" sheetId="6" r:id="rId7"/>
+    <sheet name="interactions_1" sheetId="7" r:id="rId8"/>
+    <sheet name="interactions_2" sheetId="8" r:id="rId9"/>
+    <sheet name="interactions_3" sheetId="9" r:id="rId10"/>
+    <sheet name="external_1" sheetId="10" r:id="rId11"/>
+    <sheet name="external_2" sheetId="11" r:id="rId12"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="335">
   <si>
     <t>Title</t>
   </si>
@@ -820,9 +821,6 @@
     <t>Sequenced taxa sheet name</t>
   </si>
   <si>
-    <t>SeqTaxa</t>
-  </si>
-  <si>
     <t>Reference database name</t>
   </si>
   <si>
@@ -839,13 +837,217 @@
   </si>
   <si>
     <t>https://greengenes2.ucsd.edu</t>
+  </si>
+  <si>
+    <t>Sequenced</t>
+  </si>
+  <si>
+    <t>MoreSeqData</t>
+  </si>
+  <si>
+    <t>SILVA</t>
+  </si>
+  <si>
+    <t>2024-02</t>
+  </si>
+  <si>
+    <t>Domain</t>
+  </si>
+  <si>
+    <t>Eukaryota</t>
+  </si>
+  <si>
+    <t>Fungi</t>
+  </si>
+  <si>
+    <t>Basidiomycota</t>
+  </si>
+  <si>
+    <t>Ascomycota</t>
+  </si>
+  <si>
+    <t>Mortierellomycota</t>
+  </si>
+  <si>
+    <t>Tremellomycetes</t>
+  </si>
+  <si>
+    <t>Sordariomycetes</t>
+  </si>
+  <si>
+    <t>Mortierellomycetes</t>
+  </si>
+  <si>
+    <t>Eurotiomycetes</t>
+  </si>
+  <si>
+    <t>Geoglossomycetes</t>
+  </si>
+  <si>
+    <t>Dothideomycetes</t>
+  </si>
+  <si>
+    <t>Tremellales</t>
+  </si>
+  <si>
+    <t>Hypocreales</t>
+  </si>
+  <si>
+    <t>Trichosporonales</t>
+  </si>
+  <si>
+    <t>Mortierellales</t>
+  </si>
+  <si>
+    <t>Eurotiales</t>
+  </si>
+  <si>
+    <t>Geoglossales</t>
+  </si>
+  <si>
+    <t>Pleosporales</t>
+  </si>
+  <si>
+    <t>Chaetosphaeriales</t>
+  </si>
+  <si>
+    <t>Trimorphomycetaceae</t>
+  </si>
+  <si>
+    <t>Hypocreaceae</t>
+  </si>
+  <si>
+    <t>Trichosporonaceae</t>
+  </si>
+  <si>
+    <t>Mortierellaceae</t>
+  </si>
+  <si>
+    <t>Trichocomaceae</t>
+  </si>
+  <si>
+    <t>Ophiocordycipitaceae</t>
+  </si>
+  <si>
+    <t>Geoglossaceae</t>
+  </si>
+  <si>
+    <t>Cucurbitariaceae</t>
+  </si>
+  <si>
+    <t>Clavicipitaceae</t>
+  </si>
+  <si>
+    <t>Chaetosphaeriaceae</t>
+  </si>
+  <si>
+    <t>Chloridium</t>
+  </si>
+  <si>
+    <t>Metarhizium</t>
+  </si>
+  <si>
+    <t>Trichoderma</t>
+  </si>
+  <si>
+    <t>Pyrenochaetopsis</t>
+  </si>
+  <si>
+    <t>Geoglossum</t>
+  </si>
+  <si>
+    <t>Purpureocillium</t>
+  </si>
+  <si>
+    <t>Talaromyces</t>
+  </si>
+  <si>
+    <t>Mortierella</t>
+  </si>
+  <si>
+    <t>Apiotrichum</t>
+  </si>
+  <si>
+    <t>Saitozyma</t>
+  </si>
+  <si>
+    <t>podzolica</t>
+  </si>
+  <si>
+    <t>spirale</t>
+  </si>
+  <si>
+    <t>sporotrichoides</t>
+  </si>
+  <si>
+    <t>elongata</t>
+  </si>
+  <si>
+    <t>lilacinum</t>
+  </si>
+  <si>
+    <t>harzianum</t>
+  </si>
+  <si>
+    <t>difforme</t>
+  </si>
+  <si>
+    <t>leptospora</t>
+  </si>
+  <si>
+    <t>koningiopsis</t>
+  </si>
+  <si>
+    <t>carneum</t>
+  </si>
+  <si>
+    <t>TH_100</t>
+  </si>
+  <si>
+    <t>TH_101</t>
+  </si>
+  <si>
+    <t>TH_102</t>
+  </si>
+  <si>
+    <t>TH_103</t>
+  </si>
+  <si>
+    <t>TH_104</t>
+  </si>
+  <si>
+    <t>TH_105</t>
+  </si>
+  <si>
+    <t>TH_106</t>
+  </si>
+  <si>
+    <t>TH_107</t>
+  </si>
+  <si>
+    <t>TH_108</t>
+  </si>
+  <si>
+    <t>TH_109</t>
+  </si>
+  <si>
+    <t>TH_110</t>
+  </si>
+  <si>
+    <t>TH_111</t>
+  </si>
+  <si>
+    <t>TH_113</t>
+  </si>
+  <si>
+    <t>TH_114</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -865,6 +1067,12 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -891,7 +1099,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
@@ -899,6 +1107,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1540,31 +1749,40 @@
         <v>260</v>
       </c>
       <c r="B32" t="s">
+        <v>267</v>
+      </c>
+      <c r="C32" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
         <v>261</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
+      <c r="B33" t="s">
         <v>262</v>
       </c>
-      <c r="B33" t="s">
+      <c r="C33" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
+      <c r="B34" t="s">
         <v>264</v>
       </c>
-      <c r="B34" t="s">
+      <c r="C34" s="5" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
         <v>265</v>
       </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
+      <c r="B35" s="2" t="s">
         <v>266</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>267</v>
       </c>
     </row>
   </sheetData>
@@ -1579,6 +1797,111 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68319B6E-55A5-CD40-8D21-94807C1DFFAF}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="C2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C3" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C4" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C5" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B6" t="s">
+        <v>126</v>
+      </c>
+      <c r="C6" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B7" t="s">
+        <v>129</v>
+      </c>
+      <c r="C7" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="3">
+        <v>1</v>
+      </c>
+      <c r="B8" t="s">
+        <v>132</v>
+      </c>
+      <c r="C8" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="3">
+        <v>2</v>
+      </c>
+      <c r="B9" t="s">
+        <v>135</v>
+      </c>
+      <c r="C9" t="s">
+        <v>136</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4564A69-1797-E343-B331-4E4216D5E9E0}">
   <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1734,7 +2057,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA611AD8-B75D-FF4F-B5EC-A2F06456CF6C}">
   <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -2544,6 +2867,458 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6489F378-36DF-DC49-8883-8414C559B03C}">
+  <dimension ref="A1:J15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="J1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>321</v>
+      </c>
+      <c r="B2" t="s">
+        <v>272</v>
+      </c>
+      <c r="C2" t="s">
+        <v>273</v>
+      </c>
+      <c r="D2" t="s">
+        <v>274</v>
+      </c>
+      <c r="E2" t="s">
+        <v>277</v>
+      </c>
+      <c r="F2" t="s">
+        <v>283</v>
+      </c>
+      <c r="G2" t="s">
+        <v>291</v>
+      </c>
+      <c r="H2" t="s">
+        <v>310</v>
+      </c>
+      <c r="I2" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>322</v>
+      </c>
+      <c r="B3" t="s">
+        <v>272</v>
+      </c>
+      <c r="C3" t="s">
+        <v>273</v>
+      </c>
+      <c r="D3" t="s">
+        <v>275</v>
+      </c>
+      <c r="E3" t="s">
+        <v>278</v>
+      </c>
+      <c r="F3" t="s">
+        <v>284</v>
+      </c>
+      <c r="G3" t="s">
+        <v>292</v>
+      </c>
+      <c r="H3" t="s">
+        <v>303</v>
+      </c>
+      <c r="I3" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>323</v>
+      </c>
+      <c r="B4" t="s">
+        <v>272</v>
+      </c>
+      <c r="C4" t="s">
+        <v>273</v>
+      </c>
+      <c r="D4" t="s">
+        <v>274</v>
+      </c>
+      <c r="E4" t="s">
+        <v>277</v>
+      </c>
+      <c r="F4" t="s">
+        <v>285</v>
+      </c>
+      <c r="G4" t="s">
+        <v>293</v>
+      </c>
+      <c r="H4" t="s">
+        <v>309</v>
+      </c>
+      <c r="I4" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>324</v>
+      </c>
+      <c r="B5" t="s">
+        <v>272</v>
+      </c>
+      <c r="C5" t="s">
+        <v>273</v>
+      </c>
+      <c r="D5" t="s">
+        <v>275</v>
+      </c>
+      <c r="E5" t="s">
+        <v>278</v>
+      </c>
+      <c r="F5" t="s">
+        <v>284</v>
+      </c>
+      <c r="G5" t="s">
+        <v>292</v>
+      </c>
+      <c r="H5" t="s">
+        <v>303</v>
+      </c>
+      <c r="I5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>325</v>
+      </c>
+      <c r="B6" t="s">
+        <v>272</v>
+      </c>
+      <c r="C6" t="s">
+        <v>273</v>
+      </c>
+      <c r="D6" t="s">
+        <v>276</v>
+      </c>
+      <c r="E6" t="s">
+        <v>279</v>
+      </c>
+      <c r="F6" t="s">
+        <v>286</v>
+      </c>
+      <c r="G6" t="s">
+        <v>294</v>
+      </c>
+      <c r="H6" t="s">
+        <v>308</v>
+      </c>
+      <c r="I6" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>326</v>
+      </c>
+      <c r="B7" t="s">
+        <v>272</v>
+      </c>
+      <c r="C7" t="s">
+        <v>273</v>
+      </c>
+      <c r="D7" t="s">
+        <v>275</v>
+      </c>
+      <c r="E7" t="s">
+        <v>280</v>
+      </c>
+      <c r="F7" t="s">
+        <v>287</v>
+      </c>
+      <c r="G7" t="s">
+        <v>295</v>
+      </c>
+      <c r="H7" t="s">
+        <v>307</v>
+      </c>
+      <c r="I7" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>327</v>
+      </c>
+      <c r="B8" t="s">
+        <v>272</v>
+      </c>
+      <c r="C8" t="s">
+        <v>273</v>
+      </c>
+      <c r="D8" t="s">
+        <v>275</v>
+      </c>
+      <c r="E8" t="s">
+        <v>278</v>
+      </c>
+      <c r="F8" t="s">
+        <v>284</v>
+      </c>
+      <c r="G8" t="s">
+        <v>296</v>
+      </c>
+      <c r="H8" t="s">
+        <v>306</v>
+      </c>
+      <c r="I8" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>328</v>
+      </c>
+      <c r="B9" t="s">
+        <v>272</v>
+      </c>
+      <c r="C9" t="s">
+        <v>273</v>
+      </c>
+      <c r="D9" t="s">
+        <v>275</v>
+      </c>
+      <c r="E9" t="s">
+        <v>278</v>
+      </c>
+      <c r="F9" t="s">
+        <v>284</v>
+      </c>
+      <c r="G9" t="s">
+        <v>292</v>
+      </c>
+      <c r="H9" t="s">
+        <v>303</v>
+      </c>
+      <c r="I9" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>329</v>
+      </c>
+      <c r="B10" t="s">
+        <v>272</v>
+      </c>
+      <c r="C10" t="s">
+        <v>273</v>
+      </c>
+      <c r="D10" t="s">
+        <v>275</v>
+      </c>
+      <c r="E10" t="s">
+        <v>281</v>
+      </c>
+      <c r="F10" t="s">
+        <v>288</v>
+      </c>
+      <c r="G10" t="s">
+        <v>297</v>
+      </c>
+      <c r="H10" t="s">
+        <v>305</v>
+      </c>
+      <c r="I10" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>330</v>
+      </c>
+      <c r="B11" t="s">
+        <v>272</v>
+      </c>
+      <c r="C11" t="s">
+        <v>273</v>
+      </c>
+      <c r="D11" t="s">
+        <v>275</v>
+      </c>
+      <c r="E11" t="s">
+        <v>278</v>
+      </c>
+      <c r="F11" t="s">
+        <v>284</v>
+      </c>
+      <c r="G11" t="s">
+        <v>292</v>
+      </c>
+      <c r="H11" t="s">
+        <v>303</v>
+      </c>
+      <c r="I11" t="s">
+        <v>316</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>331</v>
+      </c>
+      <c r="B12" t="s">
+        <v>272</v>
+      </c>
+      <c r="C12" t="s">
+        <v>273</v>
+      </c>
+      <c r="D12" t="s">
+        <v>275</v>
+      </c>
+      <c r="E12" t="s">
+        <v>282</v>
+      </c>
+      <c r="F12" t="s">
+        <v>289</v>
+      </c>
+      <c r="G12" t="s">
+        <v>298</v>
+      </c>
+      <c r="H12" t="s">
+        <v>304</v>
+      </c>
+      <c r="I12" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>332</v>
+      </c>
+      <c r="B13" t="s">
+        <v>272</v>
+      </c>
+      <c r="C13" t="s">
+        <v>273</v>
+      </c>
+      <c r="D13" t="s">
+        <v>275</v>
+      </c>
+      <c r="E13" t="s">
+        <v>278</v>
+      </c>
+      <c r="F13" t="s">
+        <v>284</v>
+      </c>
+      <c r="G13" t="s">
+        <v>292</v>
+      </c>
+      <c r="H13" t="s">
+        <v>303</v>
+      </c>
+      <c r="I13" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>333</v>
+      </c>
+      <c r="B14" t="s">
+        <v>272</v>
+      </c>
+      <c r="C14" t="s">
+        <v>273</v>
+      </c>
+      <c r="D14" t="s">
+        <v>275</v>
+      </c>
+      <c r="E14" t="s">
+        <v>278</v>
+      </c>
+      <c r="F14" t="s">
+        <v>284</v>
+      </c>
+      <c r="G14" t="s">
+        <v>299</v>
+      </c>
+      <c r="H14" t="s">
+        <v>302</v>
+      </c>
+      <c r="I14" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>334</v>
+      </c>
+      <c r="B15" t="s">
+        <v>272</v>
+      </c>
+      <c r="C15" t="s">
+        <v>273</v>
+      </c>
+      <c r="D15" t="s">
+        <v>275</v>
+      </c>
+      <c r="E15" t="s">
+        <v>278</v>
+      </c>
+      <c r="F15" t="s">
+        <v>290</v>
+      </c>
+      <c r="G15" t="s">
+        <v>300</v>
+      </c>
+      <c r="H15" t="s">
+        <v>301</v>
+      </c>
+      <c r="I15" t="s">
+        <v>70</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B70BB96-69CE-5C4B-B649-6188C128ED73}">
   <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -2677,7 +3452,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7FB2131-D12F-E446-A544-0D39287054FC}">
   <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -2778,7 +3553,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C9608A4-A834-0C4F-97DF-49D93E72537D}">
   <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -2894,7 +3669,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEB73AB8-5ABC-CC46-A983-918430EF84FB}">
   <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -3009,7 +3784,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7854E2C-1FBE-7947-BDF9-5436657A8287}">
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -3085,109 +3860,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68319B6E-55A5-CD40-8D21-94807C1DFFAF}">
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.6640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="B1" t="s">
-        <v>113</v>
-      </c>
-      <c r="C1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="C2" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C3" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="C4" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="B5" t="s">
-        <v>124</v>
-      </c>
-      <c r="C5" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="B6" t="s">
-        <v>126</v>
-      </c>
-      <c r="C6" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="B7" t="s">
-        <v>129</v>
-      </c>
-      <c r="C7" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" s="3">
-        <v>1</v>
-      </c>
-      <c r="B8" t="s">
-        <v>132</v>
-      </c>
-      <c r="C8" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" s="3">
-        <v>2</v>
-      </c>
-      <c r="B9" t="s">
-        <v>135</v>
-      </c>
-      <c r="C9" t="s">
-        <v>136</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Switched from using greengenes and an example link to using SILVA, as seems better maintained website
</commit_message>
<xml_diff>
--- a/docs/data_providers/data_format/Example.xlsx
+++ b/docs/data_providers/data_format/Example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jc2017/Documents/MyRepos/safedata_validator/docs/data_providers/data_format/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE15D25A-463D-3742-B77C-CB752AC55F80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25AA5BC2-253E-2249-9A5A-E6F2FA6A04C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="760" windowWidth="27360" windowHeight="16940" activeTab="3" xr2:uid="{958BE4CB-34F0-9B46-9A32-339A0F6D953C}"/>
+    <workbookView xWindow="360" yWindow="760" windowWidth="27360" windowHeight="16940" xr2:uid="{958BE4CB-34F0-9B46-9A32-339A0F6D953C}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -836,9 +836,6 @@
     <t>Reference database link</t>
   </si>
   <si>
-    <t>https://greengenes2.ucsd.edu</t>
-  </si>
-  <si>
     <t>Sequenced</t>
   </si>
   <si>
@@ -1041,6 +1038,9 @@
   </si>
   <si>
     <t>TH_114</t>
+  </si>
+  <si>
+    <t>https://www.arb-silva.de</t>
   </si>
 </sst>
 </file>
@@ -1749,10 +1749,10 @@
         <v>260</v>
       </c>
       <c r="B32" t="s">
+        <v>266</v>
+      </c>
+      <c r="C32" t="s">
         <v>267</v>
-      </c>
-      <c r="C32" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
@@ -1763,7 +1763,7 @@
         <v>262</v>
       </c>
       <c r="C33" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
@@ -1774,15 +1774,16 @@
         <v>264</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>265</v>
       </c>
-      <c r="B35" s="2" t="s">
-        <v>266</v>
+      <c r="B35" s="2"/>
+      <c r="C35" t="s">
+        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -1790,7 +1791,6 @@
     <hyperlink ref="B8" r:id="rId1" xr:uid="{8F2F57F5-1AEE-0D48-93D7-9691DA786243}"/>
     <hyperlink ref="B18" r:id="rId2" xr:uid="{854E441D-2155-F243-9B6D-EA2BAFB9B5A2}"/>
     <hyperlink ref="B22" r:id="rId3" xr:uid="{1F970723-7B44-4944-98C3-9AB1AB233E97}"/>
-    <hyperlink ref="B35" r:id="rId4" xr:uid="{3C58A218-390F-B04E-B352-36685BA79647}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2876,7 +2876,7 @@
         <v>48</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>79</v>
@@ -2905,115 +2905,115 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B2" t="s">
+        <v>271</v>
+      </c>
+      <c r="C2" t="s">
         <v>272</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>273</v>
       </c>
-      <c r="D2" t="s">
-        <v>274</v>
-      </c>
       <c r="E2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F2" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="G2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H2" t="s">
+        <v>309</v>
+      </c>
+      <c r="I2" t="s">
         <v>310</v>
-      </c>
-      <c r="I2" t="s">
-        <v>311</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B3" t="s">
+        <v>271</v>
+      </c>
+      <c r="C3" t="s">
         <v>272</v>
       </c>
-      <c r="C3" t="s">
-        <v>273</v>
-      </c>
       <c r="D3" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G3" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H3" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="I3" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B4" t="s">
+        <v>271</v>
+      </c>
+      <c r="C4" t="s">
         <v>272</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>273</v>
       </c>
-      <c r="D4" t="s">
-        <v>274</v>
-      </c>
       <c r="E4" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F4" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="G4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="H4" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="I4" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B5" t="s">
+        <v>271</v>
+      </c>
+      <c r="C5" t="s">
         <v>272</v>
       </c>
-      <c r="C5" t="s">
-        <v>273</v>
-      </c>
       <c r="D5" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E5" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G5" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H5" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="I5" t="s">
         <v>70</v>
@@ -3021,57 +3021,57 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B6" t="s">
+        <v>271</v>
+      </c>
+      <c r="C6" t="s">
         <v>272</v>
       </c>
-      <c r="C6" t="s">
-        <v>273</v>
-      </c>
       <c r="D6" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="E6" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F6" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="G6" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="H6" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="I6" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B7" t="s">
+        <v>271</v>
+      </c>
+      <c r="C7" t="s">
         <v>272</v>
       </c>
-      <c r="C7" t="s">
-        <v>273</v>
-      </c>
       <c r="D7" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E7" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F7" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="G7" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="H7" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="I7" t="s">
         <v>70</v>
@@ -3079,118 +3079,118 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B8" t="s">
+        <v>271</v>
+      </c>
+      <c r="C8" t="s">
         <v>272</v>
       </c>
-      <c r="C8" t="s">
-        <v>273</v>
-      </c>
       <c r="D8" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E8" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F8" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G8" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="H8" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="I8" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B9" t="s">
+        <v>271</v>
+      </c>
+      <c r="C9" t="s">
         <v>272</v>
       </c>
-      <c r="C9" t="s">
-        <v>273</v>
-      </c>
       <c r="D9" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E9" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F9" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G9" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H9" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="I9" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B10" t="s">
+        <v>271</v>
+      </c>
+      <c r="C10" t="s">
         <v>272</v>
       </c>
-      <c r="C10" t="s">
-        <v>273</v>
-      </c>
       <c r="D10" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E10" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="F10" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="G10" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H10" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="I10" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B11" t="s">
+        <v>271</v>
+      </c>
+      <c r="C11" t="s">
         <v>272</v>
       </c>
-      <c r="C11" t="s">
-        <v>273</v>
-      </c>
       <c r="D11" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E11" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F11" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G11" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H11" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="I11" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="J11" s="4" t="s">
         <v>243</v>
@@ -3198,115 +3198,115 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B12" t="s">
+        <v>271</v>
+      </c>
+      <c r="C12" t="s">
         <v>272</v>
       </c>
-      <c r="C12" t="s">
-        <v>273</v>
-      </c>
       <c r="D12" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E12" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="F12" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="G12" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="H12" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="I12" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B13" t="s">
+        <v>271</v>
+      </c>
+      <c r="C13" t="s">
         <v>272</v>
       </c>
-      <c r="C13" t="s">
-        <v>273</v>
-      </c>
       <c r="D13" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E13" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F13" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G13" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H13" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="I13" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="B14" t="s">
+        <v>271</v>
+      </c>
+      <c r="C14" t="s">
         <v>272</v>
       </c>
-      <c r="C14" t="s">
-        <v>273</v>
-      </c>
       <c r="D14" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E14" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F14" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H14" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="I14" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B15" t="s">
+        <v>271</v>
+      </c>
+      <c r="C15" t="s">
         <v>272</v>
       </c>
-      <c r="C15" t="s">
-        <v>273</v>
-      </c>
       <c r="D15" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E15" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F15" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G15" t="s">
+        <v>299</v>
+      </c>
+      <c r="H15" t="s">
         <v>300</v>
-      </c>
-      <c r="H15" t="s">
-        <v>301</v>
       </c>
       <c r="I15" t="s">
         <v>70</v>

</xml_diff>

<commit_message>
Removed link from Example file as that causes problems when testing using github runners
</commit_message>
<xml_diff>
--- a/docs/data_providers/data_format/Example.xlsx
+++ b/docs/data_providers/data_format/Example.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11122"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jc2017/Documents/MyRepos/safedata_validator/docs/data_providers/data_format/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jc2017/Repositories/safedata_validator/docs/data_providers/data_format/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25AA5BC2-253E-2249-9A5A-E6F2FA6A04C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6856AA7A-E42B-754B-B21D-E078E586F047}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="360" yWindow="760" windowWidth="27360" windowHeight="16940" xr2:uid="{958BE4CB-34F0-9B46-9A32-339A0F6D953C}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="335">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="579" uniqueCount="334">
   <si>
     <t>Title</t>
   </si>
@@ -1038,9 +1038,6 @@
   </si>
   <si>
     <t>TH_114</t>
-  </si>
-  <si>
-    <t>https://www.arb-silva.de</t>
   </si>
 </sst>
 </file>
@@ -1782,9 +1779,6 @@
         <v>265</v>
       </c>
       <c r="B35" s="2"/>
-      <c r="C35" t="s">
-        <v>334</v>
-      </c>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Added the safedata_validator version to the output metadata
</commit_message>
<xml_diff>
--- a/docs/data_providers/data_format/Example.xlsx
+++ b/docs/data_providers/data_format/Example.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11122"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jc2017/Repositories/safedata_validator/docs/data_providers/data_format/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6856AA7A-E42B-754B-B21D-E078E586F047}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{867250D6-FFE8-4143-9B16-3CA98B75A70E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="360" yWindow="760" windowWidth="27360" windowHeight="16940" xr2:uid="{958BE4CB-34F0-9B46-9A32-339A0F6D953C}"/>
   </bookViews>
@@ -593,9 +593,6 @@
     <t>Example worksheet showing the first method for including information from external files</t>
   </si>
   <si>
-    <t>Example worksheet showing the secod method for including information from external files</t>
-  </si>
-  <si>
     <t>Haemadipsa picta</t>
   </si>
   <si>
@@ -1038,6 +1035,9 @@
   </si>
   <si>
     <t>TH_114</t>
+  </si>
+  <si>
+    <t>Example worksheet showing the second method for including information from external files</t>
   </si>
 </sst>
 </file>
@@ -1579,7 +1579,7 @@
         <v>179</v>
       </c>
       <c r="G13" t="s">
-        <v>185</v>
+        <v>333</v>
       </c>
       <c r="H13" t="s">
         <v>184</v>
@@ -1623,10 +1623,10 @@
         <v>47</v>
       </c>
       <c r="C17" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D17" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
@@ -1743,40 +1743,40 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B32" t="s">
+        <v>265</v>
+      </c>
+      <c r="C32" t="s">
         <v>266</v>
-      </c>
-      <c r="C32" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
+        <v>260</v>
+      </c>
+      <c r="B33" t="s">
         <v>261</v>
       </c>
-      <c r="B33" t="s">
-        <v>262</v>
-      </c>
       <c r="C33" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
+        <v>262</v>
+      </c>
+      <c r="B34" t="s">
         <v>263</v>
       </c>
-      <c r="B34" t="s">
-        <v>264</v>
-      </c>
       <c r="C34" s="5" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B35" s="2"/>
     </row>
@@ -2080,7 +2080,7 @@
         <v>143</v>
       </c>
       <c r="C2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -2120,7 +2120,7 @@
         <v>147</v>
       </c>
       <c r="C7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
@@ -2380,7 +2380,7 @@
         <v>102</v>
       </c>
       <c r="B9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C9" t="s">
         <v>59</v>
@@ -2391,7 +2391,7 @@
         <v>103</v>
       </c>
       <c r="B10" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C10" t="s">
         <v>59</v>
@@ -2402,7 +2402,7 @@
         <v>131</v>
       </c>
       <c r="B11" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C11" t="s">
         <v>59</v>
@@ -2413,7 +2413,7 @@
         <v>134</v>
       </c>
       <c r="B12" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C12" t="s">
         <v>59</v>
@@ -2424,7 +2424,7 @@
         <v>132</v>
       </c>
       <c r="B13" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C13" t="s">
         <v>59</v>
@@ -2435,7 +2435,7 @@
         <v>135</v>
       </c>
       <c r="B14" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C14" t="s">
         <v>59</v>
@@ -2473,7 +2473,7 @@
         <v>81</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>73</v>
@@ -2490,103 +2490,103 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>196</v>
+      </c>
+      <c r="B2" t="s">
         <v>197</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>198</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>199</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>200</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>201</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>202</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>203</v>
-      </c>
-      <c r="H2" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>204</v>
+      </c>
+      <c r="B3" t="s">
+        <v>197</v>
+      </c>
+      <c r="C3" t="s">
         <v>205</v>
       </c>
-      <c r="B3" t="s">
-        <v>198</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>206</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>207</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>208</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>209</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>210</v>
-      </c>
-      <c r="H3" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B4" t="s">
+        <v>197</v>
+      </c>
+      <c r="C4" t="s">
+        <v>198</v>
+      </c>
+      <c r="D4" t="s">
+        <v>199</v>
+      </c>
+      <c r="E4" t="s">
         <v>212</v>
       </c>
-      <c r="B4" t="s">
-        <v>198</v>
-      </c>
-      <c r="C4" t="s">
-        <v>199</v>
-      </c>
-      <c r="D4" t="s">
-        <v>200</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>213</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>214</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>215</v>
-      </c>
-      <c r="H4" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B5" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C5" t="s">
+        <v>205</v>
+      </c>
+      <c r="D5" t="s">
         <v>206</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>207</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>208</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>209</v>
-      </c>
-      <c r="G5" t="s">
-        <v>210</v>
       </c>
       <c r="H5" t="s">
         <v>70</v>
@@ -2594,51 +2594,51 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>217</v>
+      </c>
+      <c r="B6" t="s">
+        <v>197</v>
+      </c>
+      <c r="C6" t="s">
         <v>218</v>
       </c>
-      <c r="B6" t="s">
-        <v>198</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>219</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>220</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>221</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>222</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>223</v>
-      </c>
-      <c r="H6" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>224</v>
+      </c>
+      <c r="B7" t="s">
+        <v>197</v>
+      </c>
+      <c r="C7" t="s">
+        <v>205</v>
+      </c>
+      <c r="D7" t="s">
         <v>225</v>
       </c>
-      <c r="B7" t="s">
-        <v>198</v>
-      </c>
-      <c r="C7" t="s">
-        <v>206</v>
-      </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>226</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>227</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>228</v>
-      </c>
-      <c r="G7" t="s">
-        <v>229</v>
       </c>
       <c r="H7" t="s">
         <v>70</v>
@@ -2646,210 +2646,210 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>229</v>
+      </c>
+      <c r="B8" t="s">
+        <v>197</v>
+      </c>
+      <c r="C8" t="s">
+        <v>205</v>
+      </c>
+      <c r="D8" t="s">
+        <v>206</v>
+      </c>
+      <c r="E8" t="s">
+        <v>207</v>
+      </c>
+      <c r="F8" t="s">
         <v>230</v>
       </c>
-      <c r="B8" t="s">
-        <v>198</v>
-      </c>
-      <c r="C8" t="s">
-        <v>206</v>
-      </c>
-      <c r="D8" t="s">
-        <v>207</v>
-      </c>
-      <c r="E8" t="s">
-        <v>208</v>
-      </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>231</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>232</v>
-      </c>
-      <c r="H8" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>233</v>
+      </c>
+      <c r="B9" t="s">
+        <v>197</v>
+      </c>
+      <c r="C9" t="s">
+        <v>205</v>
+      </c>
+      <c r="D9" t="s">
+        <v>206</v>
+      </c>
+      <c r="E9" t="s">
+        <v>207</v>
+      </c>
+      <c r="F9" t="s">
+        <v>208</v>
+      </c>
+      <c r="G9" t="s">
+        <v>209</v>
+      </c>
+      <c r="H9" t="s">
         <v>234</v>
-      </c>
-      <c r="B9" t="s">
-        <v>198</v>
-      </c>
-      <c r="C9" t="s">
-        <v>206</v>
-      </c>
-      <c r="D9" t="s">
-        <v>207</v>
-      </c>
-      <c r="E9" t="s">
-        <v>208</v>
-      </c>
-      <c r="F9" t="s">
-        <v>209</v>
-      </c>
-      <c r="G9" t="s">
-        <v>210</v>
-      </c>
-      <c r="H9" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>235</v>
+      </c>
+      <c r="B10" t="s">
+        <v>197</v>
+      </c>
+      <c r="C10" t="s">
+        <v>205</v>
+      </c>
+      <c r="D10" t="s">
         <v>236</v>
       </c>
-      <c r="B10" t="s">
-        <v>198</v>
-      </c>
-      <c r="C10" t="s">
-        <v>206</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>237</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>238</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>239</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>240</v>
-      </c>
-      <c r="H10" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
+        <v>241</v>
+      </c>
+      <c r="B11" t="s">
+        <v>197</v>
+      </c>
+      <c r="C11" t="s">
+        <v>205</v>
+      </c>
+      <c r="D11" t="s">
+        <v>206</v>
+      </c>
+      <c r="E11" t="s">
+        <v>207</v>
+      </c>
+      <c r="F11" t="s">
+        <v>208</v>
+      </c>
+      <c r="G11" t="s">
+        <v>209</v>
+      </c>
+      <c r="H11" t="s">
+        <v>234</v>
+      </c>
+      <c r="I11" s="4" t="s">
         <v>242</v>
-      </c>
-      <c r="B11" t="s">
-        <v>198</v>
-      </c>
-      <c r="C11" t="s">
-        <v>206</v>
-      </c>
-      <c r="D11" t="s">
-        <v>207</v>
-      </c>
-      <c r="E11" t="s">
-        <v>208</v>
-      </c>
-      <c r="F11" t="s">
-        <v>209</v>
-      </c>
-      <c r="G11" t="s">
-        <v>210</v>
-      </c>
-      <c r="H11" t="s">
-        <v>235</v>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
+        <v>243</v>
+      </c>
+      <c r="B12" t="s">
+        <v>197</v>
+      </c>
+      <c r="C12" t="s">
+        <v>205</v>
+      </c>
+      <c r="D12" t="s">
         <v>244</v>
       </c>
-      <c r="B12" t="s">
-        <v>198</v>
-      </c>
-      <c r="C12" t="s">
-        <v>206</v>
-      </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>245</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
         <v>246</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>247</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>248</v>
-      </c>
-      <c r="H12" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>249</v>
+      </c>
+      <c r="B13" t="s">
+        <v>197</v>
+      </c>
+      <c r="C13" t="s">
+        <v>205</v>
+      </c>
+      <c r="D13" t="s">
+        <v>206</v>
+      </c>
+      <c r="E13" t="s">
+        <v>207</v>
+      </c>
+      <c r="F13" t="s">
+        <v>208</v>
+      </c>
+      <c r="G13" t="s">
+        <v>209</v>
+      </c>
+      <c r="H13" t="s">
         <v>250</v>
-      </c>
-      <c r="B13" t="s">
-        <v>198</v>
-      </c>
-      <c r="C13" t="s">
-        <v>206</v>
-      </c>
-      <c r="D13" t="s">
-        <v>207</v>
-      </c>
-      <c r="E13" t="s">
-        <v>208</v>
-      </c>
-      <c r="F13" t="s">
-        <v>209</v>
-      </c>
-      <c r="G13" t="s">
-        <v>210</v>
-      </c>
-      <c r="H13" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>251</v>
+      </c>
+      <c r="B14" t="s">
+        <v>197</v>
+      </c>
+      <c r="C14" t="s">
+        <v>205</v>
+      </c>
+      <c r="D14" t="s">
+        <v>206</v>
+      </c>
+      <c r="E14" t="s">
+        <v>207</v>
+      </c>
+      <c r="F14" t="s">
         <v>252</v>
       </c>
-      <c r="B14" t="s">
-        <v>198</v>
-      </c>
-      <c r="C14" t="s">
-        <v>206</v>
-      </c>
-      <c r="D14" t="s">
-        <v>207</v>
-      </c>
-      <c r="E14" t="s">
-        <v>208</v>
-      </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>253</v>
       </c>
-      <c r="G14" t="s">
+      <c r="H14" t="s">
         <v>254</v>
-      </c>
-      <c r="H14" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
+        <v>255</v>
+      </c>
+      <c r="B15" t="s">
+        <v>197</v>
+      </c>
+      <c r="C15" t="s">
+        <v>205</v>
+      </c>
+      <c r="D15" t="s">
+        <v>206</v>
+      </c>
+      <c r="E15" t="s">
         <v>256</v>
       </c>
-      <c r="B15" t="s">
-        <v>198</v>
-      </c>
-      <c r="C15" t="s">
-        <v>206</v>
-      </c>
-      <c r="D15" t="s">
-        <v>207</v>
-      </c>
-      <c r="E15" t="s">
+      <c r="F15" t="s">
         <v>257</v>
       </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
         <v>258</v>
-      </c>
-      <c r="G15" t="s">
-        <v>259</v>
       </c>
       <c r="H15" t="s">
         <v>70</v>
@@ -2870,7 +2870,7 @@
         <v>48</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>79</v>
@@ -2882,7 +2882,7 @@
         <v>81</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>73</v>
@@ -2899,115 +2899,115 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B2" t="s">
+        <v>270</v>
+      </c>
+      <c r="C2" t="s">
         <v>271</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>272</v>
       </c>
-      <c r="D2" t="s">
-        <v>273</v>
-      </c>
       <c r="E2" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F2" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="G2" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="H2" t="s">
+        <v>308</v>
+      </c>
+      <c r="I2" t="s">
         <v>309</v>
-      </c>
-      <c r="I2" t="s">
-        <v>310</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B3" t="s">
+        <v>270</v>
+      </c>
+      <c r="C3" t="s">
         <v>271</v>
       </c>
-      <c r="C3" t="s">
-        <v>272</v>
-      </c>
       <c r="D3" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F3" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="G3" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H3" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="I3" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B4" t="s">
+        <v>270</v>
+      </c>
+      <c r="C4" t="s">
         <v>271</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>272</v>
       </c>
-      <c r="D4" t="s">
-        <v>273</v>
-      </c>
       <c r="E4" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F4" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G4" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H4" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="I4" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B5" t="s">
+        <v>270</v>
+      </c>
+      <c r="C5" t="s">
         <v>271</v>
       </c>
-      <c r="C5" t="s">
-        <v>272</v>
-      </c>
       <c r="D5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E5" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="G5" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H5" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="I5" t="s">
         <v>70</v>
@@ -3015,57 +3015,57 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B6" t="s">
+        <v>270</v>
+      </c>
+      <c r="C6" t="s">
         <v>271</v>
       </c>
-      <c r="C6" t="s">
-        <v>272</v>
-      </c>
       <c r="D6" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E6" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F6" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="G6" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="H6" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="I6" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B7" t="s">
+        <v>270</v>
+      </c>
+      <c r="C7" t="s">
         <v>271</v>
       </c>
-      <c r="C7" t="s">
-        <v>272</v>
-      </c>
       <c r="D7" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E7" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F7" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="G7" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="H7" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="I7" t="s">
         <v>70</v>
@@ -3073,234 +3073,234 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B8" t="s">
+        <v>270</v>
+      </c>
+      <c r="C8" t="s">
         <v>271</v>
       </c>
-      <c r="C8" t="s">
-        <v>272</v>
-      </c>
       <c r="D8" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E8" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F8" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="G8" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="H8" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="I8" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B9" t="s">
+        <v>270</v>
+      </c>
+      <c r="C9" t="s">
         <v>271</v>
       </c>
-      <c r="C9" t="s">
-        <v>272</v>
-      </c>
       <c r="D9" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E9" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F9" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="G9" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H9" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="I9" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B10" t="s">
+        <v>270</v>
+      </c>
+      <c r="C10" t="s">
         <v>271</v>
       </c>
-      <c r="C10" t="s">
-        <v>272</v>
-      </c>
       <c r="D10" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E10" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F10" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="G10" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="H10" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="I10" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B11" t="s">
+        <v>270</v>
+      </c>
+      <c r="C11" t="s">
         <v>271</v>
       </c>
-      <c r="C11" t="s">
-        <v>272</v>
-      </c>
       <c r="D11" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E11" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F11" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="G11" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H11" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="I11" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B12" t="s">
+        <v>270</v>
+      </c>
+      <c r="C12" t="s">
         <v>271</v>
       </c>
-      <c r="C12" t="s">
-        <v>272</v>
-      </c>
       <c r="D12" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E12" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="F12" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="G12" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H12" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="I12" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B13" t="s">
+        <v>270</v>
+      </c>
+      <c r="C13" t="s">
         <v>271</v>
       </c>
-      <c r="C13" t="s">
-        <v>272</v>
-      </c>
       <c r="D13" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E13" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F13" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="G13" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H13" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="I13" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B14" t="s">
+        <v>270</v>
+      </c>
+      <c r="C14" t="s">
         <v>271</v>
       </c>
-      <c r="C14" t="s">
-        <v>272</v>
-      </c>
       <c r="D14" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E14" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F14" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="G14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="H14" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="I14" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="B15" t="s">
+        <v>270</v>
+      </c>
+      <c r="C15" t="s">
         <v>271</v>
       </c>
-      <c r="C15" t="s">
-        <v>272</v>
-      </c>
       <c r="D15" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E15" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F15" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="G15" t="s">
+        <v>298</v>
+      </c>
+      <c r="H15" t="s">
         <v>299</v>
-      </c>
-      <c r="H15" t="s">
-        <v>300</v>
       </c>
       <c r="I15" t="s">
         <v>70</v>

</xml_diff>